<commit_message>
Update Result Test Summary
</commit_message>
<xml_diff>
--- a/Test/Test Suite/TestPlanPrincipleCommand.xlsx
+++ b/Test/Test Suite/TestPlanPrincipleCommand.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13056" tabRatio="600" firstSheet="0" activeTab="2" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="2328" windowWidth="17280" windowHeight="9420" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
@@ -15,14 +15,16 @@
     <sheet name="CommandFactory" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="7">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
+  </numFmts>
+  <fonts count="4">
     <font>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -39,27 +41,11 @@
     </font>
     <font>
       <name val="TH Sarabun New"/>
-      <family val="2"/>
-      <color theme="1"/>
-      <sz val="14"/>
-    </font>
-    <font>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <sz val="8"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <name val="TH Sarabun New"/>
       <sz val="14"/>
     </font>
     <font>
       <name val="Aptos Narrow"/>
       <sz val="14"/>
-    </font>
-    <font>
-      <name val="TH Sarabun New"/>
-      <sz val="11"/>
     </font>
   </fonts>
   <fills count="4">
@@ -82,7 +68,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="24">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -107,14 +93,16 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </left>
-      <right/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
       <top style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </top>
       <bottom style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </bottom>
       <diagonal/>
     </border>
@@ -122,90 +110,44 @@
       <left/>
       <right/>
       <top style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </top>
       <bottom style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left/>
       <right style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </right>
       <top style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </top>
       <bottom style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </left>
       <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </right>
       <top/>
       <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </bottom>
       <diagonal/>
     </border>
     <border>
       <left/>
       <right/>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
       <top style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </top>
       <bottom/>
       <diagonal/>
@@ -213,26 +155,17 @@
     <border>
       <left/>
       <right style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
       <top style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </top>
       <bottom/>
       <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </left>
       <right/>
       <top/>
@@ -241,217 +174,72 @@
     </border>
     <border>
       <left style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </left>
       <right style="thin">
-        <color indexed="64"/>
+        <color auto="1"/>
       </right>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin"/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin"/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin"/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin"/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="14" fontId="4" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -849,7 +637,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="18"/>
   <cols>
     <col width="21.77734375" bestFit="1" customWidth="1" style="2" min="1" max="1"/>
@@ -857,7 +645,9 @@
     <col width="18.109375" bestFit="1" customWidth="1" style="2" min="3" max="3"/>
     <col width="8.88671875" customWidth="1" style="2" min="4" max="5"/>
     <col width="22" bestFit="1" customWidth="1" style="2" min="6" max="6"/>
-    <col width="8.88671875" customWidth="1" style="2" min="7" max="16384"/>
+    <col width="27.21875" bestFit="1" customWidth="1" style="2" min="7" max="7"/>
+    <col width="8.88671875" customWidth="1" style="2" min="8" max="8"/>
+    <col width="8.88671875" customWidth="1" style="2" min="9" max="16384"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -885,216 +675,295 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
         <is>
           <t>SystemUnderTest</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>FunctionUnderTest</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>No of Test Cases</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
       </c>
-      <c r="E5" s="6" t="inlineStr">
+      <c r="E5" s="4" t="inlineStr">
         <is>
           <t>Fail</t>
         </is>
       </c>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="F5" s="4" t="inlineStr">
         <is>
           <t>Relative Defects (ID)</t>
         </is>
       </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>Line Coverage (%)</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="39" t="inlineStr">
+      <c r="A6" s="16" t="inlineStr">
         <is>
           <t>SendArmyCommand</t>
         </is>
       </c>
-      <c r="B6" s="39" t="inlineStr">
+      <c r="B6" s="16" t="inlineStr">
         <is>
           <t>execute</t>
         </is>
       </c>
-      <c r="C6" s="39" t="n">
+      <c r="C6" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="D6" s="39" t="n"/>
-      <c r="E6" s="39" t="n"/>
-      <c r="F6" s="39" t="n"/>
+      <c r="D6" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="E6" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="16" t="inlineStr">
+        <is>
+          <t>DEF-CMD-01</t>
+        </is>
+      </c>
+      <c r="G6" s="18" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="39" t="inlineStr">
+      <c r="A7" s="16" t="inlineStr">
         <is>
           <t>SendArmyCommand</t>
         </is>
       </c>
-      <c r="B7" s="39" t="inlineStr">
+      <c r="B7" s="16" t="inlineStr">
         <is>
           <t>getRecordedAction / getArmy</t>
         </is>
       </c>
-      <c r="C7" s="39" t="n">
+      <c r="C7" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D7" s="39" t="n"/>
-      <c r="E7" s="39" t="n"/>
-      <c r="F7" s="39" t="n"/>
+      <c r="D7" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="16" t="n"/>
+      <c r="G7" s="19" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="39" t="inlineStr">
+      <c r="A8" s="16" t="inlineStr">
         <is>
           <t>ProduceFoodCommand</t>
         </is>
       </c>
-      <c r="B8" s="39" t="inlineStr">
+      <c r="B8" s="16" t="inlineStr">
         <is>
           <t>execute</t>
         </is>
       </c>
-      <c r="C8" s="39" t="n">
+      <c r="C8" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D8" s="39" t="n"/>
-      <c r="E8" s="39" t="n"/>
-      <c r="F8" s="39" t="n"/>
+      <c r="D8" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="16" t="n"/>
+      <c r="G8" s="18" t="n">
+        <v>88.89</v>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="39" t="inlineStr">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>ProduceFoodCommand</t>
         </is>
       </c>
-      <c r="B9" s="39" t="inlineStr">
+      <c r="B9" s="16" t="inlineStr">
         <is>
           <t>getRecordedAction</t>
         </is>
       </c>
-      <c r="C9" s="39" t="n">
+      <c r="C9" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D9" s="39" t="n"/>
-      <c r="E9" s="39" t="n"/>
-      <c r="F9" s="39" t="n"/>
+      <c r="D9" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="16" t="n"/>
+      <c r="G9" s="19" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="39" t="inlineStr">
+      <c r="A10" s="16" t="inlineStr">
         <is>
           <t>RecruitSoldiersCommand</t>
         </is>
       </c>
-      <c r="B10" s="39" t="inlineStr">
+      <c r="B10" s="16" t="inlineStr">
         <is>
           <t>execute</t>
         </is>
       </c>
-      <c r="C10" s="39" t="n">
+      <c r="C10" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D10" s="39" t="n"/>
-      <c r="E10" s="39" t="n"/>
-      <c r="F10" s="39" t="n"/>
+      <c r="D10" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="16" t="n"/>
+      <c r="G10" s="18" t="n">
+        <v>88.89</v>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="39" t="inlineStr">
+      <c r="A11" s="16" t="inlineStr">
         <is>
           <t>RecruitSoldiersCommand</t>
         </is>
       </c>
-      <c r="B11" s="39" t="inlineStr">
+      <c r="B11" s="16" t="inlineStr">
         <is>
           <t>getRecordedAction</t>
         </is>
       </c>
-      <c r="C11" s="39" t="n">
+      <c r="C11" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D11" s="39" t="n"/>
-      <c r="E11" s="39" t="n"/>
-      <c r="F11" s="39" t="n"/>
+      <c r="D11" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="16" t="n"/>
+      <c r="G11" s="19" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="47" t="inlineStr">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>NoneCommand</t>
         </is>
       </c>
-      <c r="B12" s="39" t="inlineStr">
+      <c r="B12" s="16" t="inlineStr">
         <is>
           <t>execute</t>
         </is>
       </c>
-      <c r="C12" s="39" t="n">
+      <c r="C12" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D12" s="39" t="n"/>
-      <c r="E12" s="39" t="n"/>
-      <c r="F12" s="39" t="n"/>
+      <c r="D12" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="16" t="n"/>
+      <c r="G12" s="18" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="39" t="inlineStr">
+      <c r="A13" s="16" t="inlineStr">
         <is>
           <t>NoneCommand</t>
         </is>
       </c>
-      <c r="B13" s="39" t="inlineStr">
+      <c r="B13" s="16" t="inlineStr">
         <is>
           <t>getRecordedAction</t>
         </is>
       </c>
-      <c r="C13" s="39" t="n">
+      <c r="C13" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="D13" s="39" t="n"/>
-      <c r="E13" s="39" t="n"/>
-      <c r="F13" s="39" t="n"/>
+      <c r="D13" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="16" t="n"/>
+      <c r="G13" s="19" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="39" t="inlineStr">
+      <c r="A14" s="16" t="inlineStr">
         <is>
           <t>CommandFactory</t>
         </is>
       </c>
-      <c r="B14" s="39" t="inlineStr">
+      <c r="B14" s="16" t="inlineStr">
         <is>
           <t>createCommand</t>
         </is>
       </c>
-      <c r="C14" s="39" t="n">
+      <c r="C14" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="D14" s="39" t="n"/>
-      <c r="E14" s="39" t="n"/>
-      <c r="F14" s="39" t="n"/>
+      <c r="D14" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="E14" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="16" t="n"/>
+      <c r="G14" s="16" t="n">
+        <v>100</v>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="39" t="inlineStr">
+      <c r="A15" s="16" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B15" s="50" t="n"/>
-      <c r="C15" s="39" t="n">
+      <c r="B15" s="17" t="n"/>
+      <c r="C15" s="16" t="n">
         <v>17</v>
       </c>
-      <c r="D15" s="41" t="n"/>
-      <c r="E15" s="41" t="n"/>
-      <c r="F15" s="41" t="n"/>
+      <c r="D15" s="24" t="n">
+        <v>17</v>
+      </c>
+      <c r="E15" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="24" t="inlineStr">
+        <is>
+          <t>DEF-CMD-01</t>
+        </is>
+      </c>
+      <c r="G15" s="24" t="n">
+        <v>96.55</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="5">
     <mergeCell ref="A15:B15"/>
+    <mergeCell ref="G8:G9"/>
+    <mergeCell ref="G12:G13"/>
+    <mergeCell ref="G6:G7"/>
+    <mergeCell ref="G10:G11"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1111,10 +980,10 @@
   <cols>
     <col width="4.33203125" bestFit="1" customWidth="1" style="2" min="1" max="1"/>
     <col width="9.88671875" bestFit="1" customWidth="1" style="2" min="2" max="2"/>
-    <col width="12" bestFit="1" customWidth="1" style="2" min="3" max="3"/>
-    <col width="12.77734375" bestFit="1" customWidth="1" style="2" min="4" max="4"/>
-    <col width="8.21875" bestFit="1" customWidth="1" style="2" min="5" max="5"/>
-    <col width="13.21875" bestFit="1" customWidth="1" style="2" min="6" max="6"/>
+    <col width="30" bestFit="1" customWidth="1" style="2" min="3" max="3"/>
+    <col width="52" bestFit="1" customWidth="1" style="2" min="4" max="4"/>
+    <col width="60" bestFit="1" customWidth="1" style="2" min="5" max="5"/>
+    <col width="13" bestFit="1" customWidth="1" style="2" min="6" max="6"/>
     <col width="34.44140625" bestFit="1" customWidth="1" style="2" min="7" max="7"/>
   </cols>
   <sheetData>
@@ -1155,16 +1024,38 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="72" customHeight="1">
       <c r="A2" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="n"/>
-      <c r="C2" s="3" t="n"/>
-      <c r="D2" s="3" t="n"/>
-      <c r="E2" s="3" t="n"/>
-      <c r="F2" s="3" t="n"/>
-      <c r="G2" s="3" t="n"/>
+      <c r="B2" s="12" t="inlineStr">
+        <is>
+          <t>DEF-CMD-01</t>
+        </is>
+      </c>
+      <c r="C2" s="13" t="inlineStr">
+        <is>
+          <t>Rebellion branch cannot be forced deterministically</t>
+        </is>
+      </c>
+      <c r="D2" s="13" t="inlineStr">
+        <is>
+          <t>SendArmyCommand TC04 asks for the 20% rebellion branch to be forced, but the check calls ThreadLocalRandom directly and the class has no injectable seam.</t>
+        </is>
+      </c>
+      <c r="E2" s="13" t="inlineStr">
+        <is>
+          <t>SendArmyCommand.java:44-51. Workaround: 300 executions and an assertion that both branches appeared, with per-attempt effects checked on each rebellion. A fix is an injectable Random or a strategy object.</t>
+        </is>
+      </c>
+      <c r="F2" s="14" t="n">
+        <v>46305</v>
+      </c>
+      <c r="G2" s="13" t="inlineStr">
+        <is>
+          <t>Opened</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="n">
@@ -1222,286 +1113,337 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A3:G17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="46" customWidth="1" min="3" max="3"/>
-    <col width="46" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="3" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="3">
-      <c r="A3" s="42" t="inlineStr">
+    <row r="3" ht="42" customHeight="1">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>Project Name</t>
         </is>
       </c>
-      <c r="B3" s="43" t="inlineStr">
+      <c r="B3" s="20" t="inlineStr">
         <is>
           <t>Eternal Crash2</t>
         </is>
       </c>
-      <c r="C3" s="51" t="n"/>
-      <c r="D3" s="51" t="n"/>
-      <c r="E3" s="51" t="n"/>
-      <c r="F3" s="51" t="n"/>
-      <c r="G3" s="50" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="42" t="inlineStr">
+      <c r="C3" s="21" t="n"/>
+      <c r="D3" s="21" t="n"/>
+      <c r="E3" s="21" t="n"/>
+      <c r="F3" s="21" t="n"/>
+      <c r="G3" s="17" t="n"/>
+    </row>
+    <row r="4" ht="84" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>SystemUnderTest/Class under Test</t>
         </is>
       </c>
-      <c r="B4" s="43" t="inlineStr">
+      <c r="B4" s="20" t="inlineStr">
         <is>
           <t>SendArmyCommand</t>
         </is>
       </c>
-      <c r="C4" s="51" t="n"/>
-      <c r="D4" s="51" t="n"/>
-      <c r="E4" s="51" t="n"/>
-      <c r="F4" s="51" t="n"/>
-      <c r="G4" s="50" t="n"/>
+      <c r="C4" s="21" t="n"/>
+      <c r="D4" s="21" t="n"/>
+      <c r="E4" s="21" t="n"/>
+      <c r="F4" s="21" t="n"/>
+      <c r="G4" s="17" t="n"/>
     </row>
     <row r="5" ht="35.4" customHeight="1">
-      <c r="A5" s="42" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>Environment</t>
         </is>
       </c>
-      <c r="B5" s="43" t="inlineStr">
-        <is>
-          <t>Window 11, java version "1.8.0_503" , Junit 5</t>
-        </is>
-      </c>
-      <c r="C5" s="51" t="n"/>
-      <c r="D5" s="51" t="n"/>
-      <c r="E5" s="51" t="n"/>
-      <c r="F5" s="51" t="n"/>
-      <c r="G5" s="50" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="42" t="inlineStr">
+      <c r="B5" s="20" t="inlineStr">
+        <is>
+          <t>Window 11, java version "17.0.12" , Junit 5</t>
+        </is>
+      </c>
+      <c r="C5" s="21" t="n"/>
+      <c r="D5" s="21" t="n"/>
+      <c r="E5" s="21" t="n"/>
+      <c r="F5" s="21" t="n"/>
+      <c r="G5" s="17" t="n"/>
+    </row>
+    <row r="6" ht="21" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B6" s="45" t="n">
+      <c r="B6" s="23" t="n">
         <v>46305</v>
       </c>
-      <c r="C6" s="51" t="n"/>
-      <c r="D6" s="51" t="n"/>
-      <c r="E6" s="51" t="n"/>
-      <c r="F6" s="51" t="n"/>
-      <c r="G6" s="50" t="n"/>
+      <c r="C6" s="21" t="n"/>
+      <c r="D6" s="21" t="n"/>
+      <c r="E6" s="21" t="n"/>
+      <c r="F6" s="21" t="n"/>
+      <c r="G6" s="17" t="n"/>
     </row>
     <row r="7" ht="35.4" customHeight="1">
-      <c r="A7" s="42" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>Requirement</t>
         </is>
       </c>
-      <c r="B7" s="46" t="inlineStr">
+      <c r="B7" s="22" t="inlineStr">
         <is>
           <t>Mock ArmyService, GameEventRepository; real City/Player/Game builders</t>
         </is>
       </c>
-      <c r="C7" s="51" t="n"/>
-      <c r="D7" s="51" t="n"/>
-      <c r="E7" s="51" t="n"/>
-      <c r="F7" s="51" t="n"/>
-      <c r="G7" s="50" t="n"/>
+      <c r="C7" s="21" t="n"/>
+      <c r="D7" s="21" t="n"/>
+      <c r="E7" s="21" t="n"/>
+      <c r="F7" s="21" t="n"/>
+      <c r="G7" s="17" t="n"/>
     </row>
     <row r="11" ht="21" customHeight="1">
-      <c r="A11" s="43" t="inlineStr">
+      <c r="A11" s="20" t="inlineStr">
         <is>
           <t>TestCaseID</t>
         </is>
       </c>
-      <c r="B11" s="43" t="inlineStr">
+      <c r="B11" s="20" t="inlineStr">
         <is>
           <t>Function Under Test</t>
         </is>
       </c>
-      <c r="C11" s="43" t="inlineStr">
+      <c r="C11" s="20" t="inlineStr">
         <is>
           <t>TestData</t>
         </is>
       </c>
-      <c r="D11" s="43" t="inlineStr">
+      <c r="D11" s="20" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="E11" s="43" t="inlineStr">
+      <c r="E11" s="20" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="F11" s="43" t="inlineStr">
+      <c r="F11" s="20" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="G11" s="43" t="inlineStr">
+      <c r="G11" s="20" t="inlineStr">
         <is>
           <t>DefectID</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="43" t="inlineStr">
+    <row r="12" ht="54" customHeight="1">
+      <c r="A12" s="20" t="inlineStr">
         <is>
           <t>TC01</t>
         </is>
       </c>
-      <c r="B12" s="43" t="inlineStr">
+      <c r="B12" s="20" t="inlineStr">
         <is>
           <t>execute</t>
         </is>
       </c>
-      <c r="C12" s="46" t="inlineStr">
+      <c r="C12" s="22" t="inlineStr">
         <is>
           <t>SendArmyCommand(armyService, City(id10, player100), targetCityId 20, soldierCount 20, turn 1)</t>
         </is>
       </c>
-      <c r="D12" s="46" t="inlineStr">
+      <c r="D12" s="22" t="inlineStr">
         <is>
           <t>verify(armyService).sendArmy(10L, 20L, 20, 1)</t>
         </is>
       </c>
-      <c r="E12" s="43" t="n"/>
-      <c r="F12" s="43" t="n"/>
-      <c r="G12" s="43" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="43" t="inlineStr">
+      <c r="E12" s="15" t="inlineStr">
+        <is>
+          <t>armyService.sendArmy(10L, 20L, 20, 1) called exactly once</t>
+        </is>
+      </c>
+      <c r="F12" s="20" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G12" s="20" t="n"/>
+    </row>
+    <row r="13" ht="72" customHeight="1">
+      <c r="A13" s="20" t="inlineStr">
         <is>
           <t>TC02</t>
         </is>
       </c>
-      <c r="B13" s="43" t="inlineStr">
+      <c r="B13" s="20" t="inlineStr">
         <is>
           <t>execute</t>
         </is>
       </c>
-      <c r="C13" s="46" t="inlineStr">
+      <c r="C13" s="22" t="inlineStr">
         <is>
           <t>targetCityId = null</t>
         </is>
       </c>
-      <c r="D13" s="46" t="inlineStr">
+      <c r="D13" s="22" t="inlineStr">
         <is>
           <t>throws BusinessLogicException 'Target and soldier count are required to send an army'; armyService never called</t>
         </is>
       </c>
-      <c r="E13" s="43" t="n"/>
-      <c r="F13" s="43" t="n"/>
-      <c r="G13" s="43" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="43" t="inlineStr">
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>BusinessLogicException 'Target and soldier count are required to send an army'; no interaction with armyService or gameEventRepository</t>
+        </is>
+      </c>
+      <c r="F13" s="20" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G13" s="20" t="n"/>
+    </row>
+    <row r="14" ht="36" customHeight="1">
+      <c r="A14" s="20" t="inlineStr">
         <is>
           <t>TC03</t>
         </is>
       </c>
-      <c r="B14" s="43" t="inlineStr">
+      <c r="B14" s="20" t="inlineStr">
         <is>
           <t>execute</t>
         </is>
       </c>
-      <c r="C14" s="46" t="inlineStr">
+      <c r="C14" s="22" t="inlineStr">
         <is>
           <t>soldierCount = null</t>
         </is>
       </c>
-      <c r="D14" s="46" t="inlineStr">
+      <c r="D14" s="22" t="inlineStr">
         <is>
           <t>same BusinessLogicException</t>
         </is>
       </c>
-      <c r="E14" s="43" t="n"/>
-      <c r="F14" s="43" t="n"/>
-      <c r="G14" s="43" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="43" t="inlineStr">
+      <c r="E14" s="15" t="inlineStr">
+        <is>
+          <t>the same BusinessLogicException message; nothing sent and no event written</t>
+        </is>
+      </c>
+      <c r="F14" s="20" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G14" s="20" t="n"/>
+    </row>
+    <row r="15" ht="144" customHeight="1">
+      <c r="A15" s="20" t="inlineStr">
         <is>
           <t>TC04</t>
         </is>
       </c>
-      <c r="B15" s="43" t="inlineStr">
+      <c r="B15" s="20" t="inlineStr">
         <is>
           <t>execute</t>
         </is>
       </c>
-      <c r="C15" s="46" t="inlineStr">
+      <c r="C15" s="22" t="inlineStr">
         <is>
           <t>owner has Marshal(specialAbilityType 'SURVIVE_DESTRUCTION') (force the 20% branch)</t>
         </is>
       </c>
-      <c r="D15" s="46" t="inlineStr">
+      <c r="D15" s="22" t="inlineStr">
         <is>
           <t>armyService.sendArmy NOT called; recordedAction == NONE; sourceCity.actionUsedThisTurn == true; REBELLION GameEvent saved</t>
         </is>
       </c>
-      <c r="E15" s="43" t="n"/>
-      <c r="F15" s="43" t="n"/>
-      <c r="G15" s="43" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="43" t="inlineStr">
+      <c r="E15" s="15" t="inlineStr">
+        <is>
+          <t>the 20% rebellion roll has no injection seam, so 300 executions were run: on every rebellion attempt armyService.sendArmy was not called, recordedAction was NONE and the source city consumed its action, while the remaining attempts sent the army normally; one REBELLION GameEvent per rebellion, affected by the owner</t>
+        </is>
+      </c>
+      <c r="F15" s="20" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G15" s="20" t="inlineStr">
+        <is>
+          <t>DEF-CMD-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="54" customHeight="1">
+      <c r="A16" s="20" t="inlineStr">
         <is>
           <t>TC05</t>
         </is>
       </c>
-      <c r="B16" s="43" t="inlineStr">
+      <c r="B16" s="20" t="inlineStr">
         <is>
           <t>execute</t>
         </is>
       </c>
-      <c r="C16" s="46" t="inlineStr">
+      <c r="C16" s="22" t="inlineStr">
         <is>
           <t>owner has Marshal(revealsAttackTarget = true), normal send</t>
         </is>
       </c>
-      <c r="D16" s="46" t="inlineStr">
+      <c r="D16" s="22" t="inlineStr">
         <is>
           <t>army sent AND a REBELLION 'declaration of war' GameEvent saved against the target city's owner</t>
         </is>
       </c>
-      <c r="E16" s="43" t="n"/>
-      <c r="F16" s="43" t="n"/>
-      <c r="G16" s="43" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="43" t="inlineStr">
+      <c r="E16" s="15" t="inlineStr">
+        <is>
+          <t>army sent and 1 REBELLION event saved with the target city's owner as affectedPlayer and 'City-20' in the description</t>
+        </is>
+      </c>
+      <c r="F16" s="20" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G16" s="20" t="n"/>
+    </row>
+    <row r="17" ht="54" customHeight="1">
+      <c r="A17" s="20" t="inlineStr">
         <is>
           <t>TC06</t>
         </is>
       </c>
-      <c r="B17" s="43" t="inlineStr">
+      <c r="B17" s="20" t="inlineStr">
         <is>
           <t>getRecordedAction / getArmy</t>
         </is>
       </c>
-      <c r="C17" s="46" t="inlineStr">
+      <c r="C17" s="22" t="inlineStr">
         <is>
           <t>after a normal execute()</t>
         </is>
       </c>
-      <c r="D17" s="46" t="inlineStr">
+      <c r="D17" s="22" t="inlineStr">
         <is>
           <t>recordedAction == SEND_ARMY; getArmy() returns the army returned by armyService.sendArmy</t>
         </is>
       </c>
-      <c r="E17" s="43" t="n"/>
-      <c r="F17" s="43" t="n"/>
-      <c r="G17" s="43" t="n"/>
+      <c r="E17" s="15" t="inlineStr">
+        <is>
+          <t>recordedAction == SEND_ARMY, getArmy() returns the army from armyService.sendArmy, no GameEvent written</t>
+        </is>
+      </c>
+      <c r="F17" s="20" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G17" s="20" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -1522,186 +1464,201 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A3:G13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="46" customWidth="1" min="3" max="3"/>
-    <col width="46" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="3" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="3">
-      <c r="A3" s="44" t="inlineStr">
+    <row r="3" ht="21" customHeight="1">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>Project Name</t>
         </is>
       </c>
-      <c r="B3" s="41" t="inlineStr">
+      <c r="B3" s="24" t="inlineStr">
         <is>
           <t>Eternal Crash2</t>
         </is>
       </c>
-      <c r="C3" s="51" t="n"/>
-      <c r="D3" s="51" t="n"/>
-      <c r="E3" s="51" t="n"/>
-      <c r="F3" s="51" t="n"/>
-      <c r="G3" s="50" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="44" t="inlineStr">
+      <c r="C3" s="21" t="n"/>
+      <c r="D3" s="21" t="n"/>
+      <c r="E3" s="21" t="n"/>
+      <c r="F3" s="21" t="n"/>
+      <c r="G3" s="17" t="n"/>
+    </row>
+    <row r="4" ht="21" customHeight="1">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>SystemUnderTest/Class under Test</t>
         </is>
       </c>
-      <c r="B4" s="41" t="inlineStr">
+      <c r="B4" s="24" t="inlineStr">
         <is>
           <t>ProduceFoodCommand</t>
         </is>
       </c>
-      <c r="C4" s="51" t="n"/>
-      <c r="D4" s="51" t="n"/>
-      <c r="E4" s="51" t="n"/>
-      <c r="F4" s="51" t="n"/>
-      <c r="G4" s="50" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="44" t="inlineStr">
+      <c r="C4" s="21" t="n"/>
+      <c r="D4" s="21" t="n"/>
+      <c r="E4" s="21" t="n"/>
+      <c r="F4" s="21" t="n"/>
+      <c r="G4" s="17" t="n"/>
+    </row>
+    <row r="5" ht="21" customHeight="1">
+      <c r="A5" s="9" t="inlineStr">
         <is>
           <t>Environment</t>
         </is>
       </c>
-      <c r="B5" s="41" t="inlineStr">
-        <is>
-          <t>Window 11, java version "1.8.0_503" , Junit 5</t>
-        </is>
-      </c>
-      <c r="C5" s="51" t="n"/>
-      <c r="D5" s="51" t="n"/>
-      <c r="E5" s="51" t="n"/>
-      <c r="F5" s="51" t="n"/>
-      <c r="G5" s="50" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="44" t="inlineStr">
+      <c r="B5" s="24" t="inlineStr">
+        <is>
+          <t>Window 11, java version "17.0.12" , Junit 5</t>
+        </is>
+      </c>
+      <c r="C5" s="21" t="n"/>
+      <c r="D5" s="21" t="n"/>
+      <c r="E5" s="21" t="n"/>
+      <c r="F5" s="21" t="n"/>
+      <c r="G5" s="17" t="n"/>
+    </row>
+    <row r="6" ht="21" customHeight="1">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B6" s="49" t="n">
+      <c r="B6" s="25" t="n">
         <v>46305</v>
       </c>
-      <c r="C6" s="51" t="n"/>
-      <c r="D6" s="51" t="n"/>
-      <c r="E6" s="51" t="n"/>
-      <c r="F6" s="51" t="n"/>
-      <c r="G6" s="50" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="44" t="inlineStr">
+      <c r="C6" s="21" t="n"/>
+      <c r="D6" s="21" t="n"/>
+      <c r="E6" s="21" t="n"/>
+      <c r="F6" s="21" t="n"/>
+      <c r="G6" s="17" t="n"/>
+    </row>
+    <row r="7" ht="21" customHeight="1">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>Requirement</t>
         </is>
       </c>
-      <c r="B7" s="41" t="inlineStr">
+      <c r="B7" s="24" t="inlineStr">
         <is>
           <t>Mock CityService</t>
         </is>
       </c>
-      <c r="C7" s="51" t="n"/>
-      <c r="D7" s="51" t="n"/>
-      <c r="E7" s="51" t="n"/>
-      <c r="F7" s="51" t="n"/>
-      <c r="G7" s="50" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="43" t="inlineStr">
+      <c r="C7" s="21" t="n"/>
+      <c r="D7" s="21" t="n"/>
+      <c r="E7" s="21" t="n"/>
+      <c r="F7" s="21" t="n"/>
+      <c r="G7" s="17" t="n"/>
+    </row>
+    <row r="11" ht="21" customHeight="1">
+      <c r="A11" s="20" t="inlineStr">
         <is>
           <t>TestCaseID</t>
         </is>
       </c>
-      <c r="B11" s="43" t="inlineStr">
+      <c r="B11" s="20" t="inlineStr">
         <is>
           <t>Function Under Test</t>
         </is>
       </c>
-      <c r="C11" s="43" t="inlineStr">
+      <c r="C11" s="20" t="inlineStr">
         <is>
           <t>TestData</t>
         </is>
       </c>
-      <c r="D11" s="43" t="inlineStr">
+      <c r="D11" s="20" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="E11" s="43" t="inlineStr">
+      <c r="E11" s="20" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="F11" s="43" t="inlineStr">
+      <c r="F11" s="20" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="G11" s="43" t="inlineStr">
+      <c r="G11" s="20" t="inlineStr">
         <is>
           <t>DefectID</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="43" t="inlineStr">
+    <row r="12" ht="36" customHeight="1">
+      <c r="A12" s="20" t="inlineStr">
         <is>
           <t>TC01</t>
         </is>
       </c>
-      <c r="B12" s="43" t="inlineStr">
+      <c r="B12" s="20" t="inlineStr">
         <is>
           <t>execute</t>
         </is>
       </c>
-      <c r="C12" s="46" t="inlineStr">
+      <c r="C12" s="22" t="inlineStr">
         <is>
           <t>ProduceFoodCommand(cityService, 10L, 1).execute()</t>
         </is>
       </c>
-      <c r="D12" s="46" t="inlineStr">
+      <c r="D12" s="22" t="inlineStr">
         <is>
           <t>verify(cityService).produceFood(10L, 1)</t>
         </is>
       </c>
-      <c r="E12" s="43" t="n"/>
-      <c r="F12" s="43" t="n"/>
-      <c r="G12" s="43" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="43" t="inlineStr">
+      <c r="E12" s="15" t="inlineStr">
+        <is>
+          <t>cityService.produceFood(10L, 1) called exactly once</t>
+        </is>
+      </c>
+      <c r="F12" s="20" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G12" s="20" t="n"/>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="20" t="inlineStr">
         <is>
           <t>TC02</t>
         </is>
       </c>
-      <c r="B13" s="43" t="inlineStr">
+      <c r="B13" s="20" t="inlineStr">
         <is>
           <t>getRecordedAction</t>
         </is>
       </c>
-      <c r="C13" s="46" t="inlineStr">
+      <c r="C13" s="22" t="inlineStr">
         <is>
           <t>any instance</t>
         </is>
       </c>
-      <c r="D13" s="46" t="inlineStr">
+      <c r="D13" s="22" t="inlineStr">
         <is>
           <t>ActionType.PRODUCE_FOOD</t>
         </is>
       </c>
-      <c r="E13" s="43" t="n"/>
-      <c r="F13" s="43" t="n"/>
-      <c r="G13" s="43" t="n"/>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>ActionType.PRODUCE_FOOD</t>
+        </is>
+      </c>
+      <c r="F13" s="20" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G13" s="20" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -1722,186 +1679,201 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A3:G13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="46" customWidth="1" min="3" max="3"/>
-    <col width="46" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="3" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="3">
-      <c r="A3" s="44" t="inlineStr">
+    <row r="3" ht="21" customHeight="1">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>Project Name</t>
         </is>
       </c>
-      <c r="B3" s="41" t="inlineStr">
+      <c r="B3" s="24" t="inlineStr">
         <is>
           <t>Eternal Crash2</t>
         </is>
       </c>
-      <c r="C3" s="51" t="n"/>
-      <c r="D3" s="51" t="n"/>
-      <c r="E3" s="51" t="n"/>
-      <c r="F3" s="51" t="n"/>
-      <c r="G3" s="50" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="44" t="inlineStr">
+      <c r="C3" s="21" t="n"/>
+      <c r="D3" s="21" t="n"/>
+      <c r="E3" s="21" t="n"/>
+      <c r="F3" s="21" t="n"/>
+      <c r="G3" s="17" t="n"/>
+    </row>
+    <row r="4" ht="21" customHeight="1">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>SystemUnderTest/Class under Test</t>
         </is>
       </c>
-      <c r="B4" s="41" t="inlineStr">
+      <c r="B4" s="24" t="inlineStr">
         <is>
           <t>RecruitSoldiersCommand</t>
         </is>
       </c>
-      <c r="C4" s="51" t="n"/>
-      <c r="D4" s="51" t="n"/>
-      <c r="E4" s="51" t="n"/>
-      <c r="F4" s="51" t="n"/>
-      <c r="G4" s="50" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="44" t="inlineStr">
+      <c r="C4" s="21" t="n"/>
+      <c r="D4" s="21" t="n"/>
+      <c r="E4" s="21" t="n"/>
+      <c r="F4" s="21" t="n"/>
+      <c r="G4" s="17" t="n"/>
+    </row>
+    <row r="5" ht="21" customHeight="1">
+      <c r="A5" s="9" t="inlineStr">
         <is>
           <t>Environment</t>
         </is>
       </c>
-      <c r="B5" s="41" t="inlineStr">
-        <is>
-          <t>Window 11, java version "1.8.0_503" , Junit 5</t>
-        </is>
-      </c>
-      <c r="C5" s="51" t="n"/>
-      <c r="D5" s="51" t="n"/>
-      <c r="E5" s="51" t="n"/>
-      <c r="F5" s="51" t="n"/>
-      <c r="G5" s="50" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="44" t="inlineStr">
+      <c r="B5" s="24" t="inlineStr">
+        <is>
+          <t>Window 11, java version "17.0.12" , Junit 5</t>
+        </is>
+      </c>
+      <c r="C5" s="21" t="n"/>
+      <c r="D5" s="21" t="n"/>
+      <c r="E5" s="21" t="n"/>
+      <c r="F5" s="21" t="n"/>
+      <c r="G5" s="17" t="n"/>
+    </row>
+    <row r="6" ht="21" customHeight="1">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B6" s="49" t="n">
+      <c r="B6" s="25" t="n">
         <v>46305</v>
       </c>
-      <c r="C6" s="51" t="n"/>
-      <c r="D6" s="51" t="n"/>
-      <c r="E6" s="51" t="n"/>
-      <c r="F6" s="51" t="n"/>
-      <c r="G6" s="50" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="44" t="inlineStr">
+      <c r="C6" s="21" t="n"/>
+      <c r="D6" s="21" t="n"/>
+      <c r="E6" s="21" t="n"/>
+      <c r="F6" s="21" t="n"/>
+      <c r="G6" s="17" t="n"/>
+    </row>
+    <row r="7" ht="21" customHeight="1">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>Requirement</t>
         </is>
       </c>
-      <c r="B7" s="41" t="inlineStr">
+      <c r="B7" s="24" t="inlineStr">
         <is>
           <t>Mock CityService</t>
         </is>
       </c>
-      <c r="C7" s="51" t="n"/>
-      <c r="D7" s="51" t="n"/>
-      <c r="E7" s="51" t="n"/>
-      <c r="F7" s="51" t="n"/>
-      <c r="G7" s="50" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="43" t="inlineStr">
+      <c r="C7" s="21" t="n"/>
+      <c r="D7" s="21" t="n"/>
+      <c r="E7" s="21" t="n"/>
+      <c r="F7" s="21" t="n"/>
+      <c r="G7" s="17" t="n"/>
+    </row>
+    <row r="11" ht="21" customHeight="1">
+      <c r="A11" s="20" t="inlineStr">
         <is>
           <t>TestCaseID</t>
         </is>
       </c>
-      <c r="B11" s="43" t="inlineStr">
+      <c r="B11" s="20" t="inlineStr">
         <is>
           <t>Function Under Test</t>
         </is>
       </c>
-      <c r="C11" s="43" t="inlineStr">
+      <c r="C11" s="20" t="inlineStr">
         <is>
           <t>TestData</t>
         </is>
       </c>
-      <c r="D11" s="43" t="inlineStr">
+      <c r="D11" s="20" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="E11" s="43" t="inlineStr">
+      <c r="E11" s="20" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="F11" s="43" t="inlineStr">
+      <c r="F11" s="20" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="G11" s="43" t="inlineStr">
+      <c r="G11" s="20" t="inlineStr">
         <is>
           <t>DefectID</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="43" t="inlineStr">
+    <row r="12" ht="36" customHeight="1">
+      <c r="A12" s="20" t="inlineStr">
         <is>
           <t>TC01</t>
         </is>
       </c>
-      <c r="B12" s="43" t="inlineStr">
+      <c r="B12" s="20" t="inlineStr">
         <is>
           <t>execute</t>
         </is>
       </c>
-      <c r="C12" s="46" t="inlineStr">
+      <c r="C12" s="22" t="inlineStr">
         <is>
           <t>RecruitSoldiersCommand(cityService, 10L, 6).execute()</t>
         </is>
       </c>
-      <c r="D12" s="46" t="inlineStr">
+      <c r="D12" s="22" t="inlineStr">
         <is>
           <t>verify(cityService).recruitSoldiers(10L, 6)</t>
         </is>
       </c>
-      <c r="E12" s="43" t="n"/>
-      <c r="F12" s="43" t="n"/>
-      <c r="G12" s="43" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="43" t="inlineStr">
+      <c r="E12" s="15" t="inlineStr">
+        <is>
+          <t>cityService.recruitSoldiers(10L, 6) called exactly once</t>
+        </is>
+      </c>
+      <c r="F12" s="20" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G12" s="20" t="n"/>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="20" t="inlineStr">
         <is>
           <t>TC02</t>
         </is>
       </c>
-      <c r="B13" s="43" t="inlineStr">
+      <c r="B13" s="20" t="inlineStr">
         <is>
           <t>getRecordedAction</t>
         </is>
       </c>
-      <c r="C13" s="46" t="inlineStr">
+      <c r="C13" s="22" t="inlineStr">
         <is>
           <t>any instance</t>
         </is>
       </c>
-      <c r="D13" s="46" t="inlineStr">
+      <c r="D13" s="22" t="inlineStr">
         <is>
           <t>ActionType.RECRUIT_SOLDIERS</t>
         </is>
       </c>
-      <c r="E13" s="43" t="n"/>
-      <c r="F13" s="43" t="n"/>
-      <c r="G13" s="43" t="n"/>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>ActionType.RECRUIT_SOLDIERS</t>
+        </is>
+      </c>
+      <c r="F13" s="20" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G13" s="20" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -1922,186 +1894,201 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A3:G13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="46" customWidth="1" min="3" max="3"/>
-    <col width="46" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="3" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="3">
-      <c r="A3" s="44" t="inlineStr">
+    <row r="3" ht="21" customHeight="1">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>Project Name</t>
         </is>
       </c>
-      <c r="B3" s="41" t="inlineStr">
+      <c r="B3" s="24" t="inlineStr">
         <is>
           <t>Eternal Crash2</t>
         </is>
       </c>
-      <c r="C3" s="51" t="n"/>
-      <c r="D3" s="51" t="n"/>
-      <c r="E3" s="51" t="n"/>
-      <c r="F3" s="51" t="n"/>
-      <c r="G3" s="50" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="44" t="inlineStr">
+      <c r="C3" s="21" t="n"/>
+      <c r="D3" s="21" t="n"/>
+      <c r="E3" s="21" t="n"/>
+      <c r="F3" s="21" t="n"/>
+      <c r="G3" s="17" t="n"/>
+    </row>
+    <row r="4" ht="21" customHeight="1">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>SystemUnderTest/Class under Test</t>
         </is>
       </c>
-      <c r="B4" s="41" t="inlineStr">
+      <c r="B4" s="24" t="inlineStr">
         <is>
           <t>NoneCommand</t>
         </is>
       </c>
-      <c r="C4" s="51" t="n"/>
-      <c r="D4" s="51" t="n"/>
-      <c r="E4" s="51" t="n"/>
-      <c r="F4" s="51" t="n"/>
-      <c r="G4" s="50" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="44" t="inlineStr">
+      <c r="C4" s="21" t="n"/>
+      <c r="D4" s="21" t="n"/>
+      <c r="E4" s="21" t="n"/>
+      <c r="F4" s="21" t="n"/>
+      <c r="G4" s="17" t="n"/>
+    </row>
+    <row r="5" ht="21" customHeight="1">
+      <c r="A5" s="9" t="inlineStr">
         <is>
           <t>Environment</t>
         </is>
       </c>
-      <c r="B5" s="41" t="inlineStr">
-        <is>
-          <t>Window 11, java version "1.8.0_503" , Junit 5</t>
-        </is>
-      </c>
-      <c r="C5" s="51" t="n"/>
-      <c r="D5" s="51" t="n"/>
-      <c r="E5" s="51" t="n"/>
-      <c r="F5" s="51" t="n"/>
-      <c r="G5" s="50" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="44" t="inlineStr">
+      <c r="B5" s="24" t="inlineStr">
+        <is>
+          <t>Window 11, java version "17.0.12" , Junit 5</t>
+        </is>
+      </c>
+      <c r="C5" s="21" t="n"/>
+      <c r="D5" s="21" t="n"/>
+      <c r="E5" s="21" t="n"/>
+      <c r="F5" s="21" t="n"/>
+      <c r="G5" s="17" t="n"/>
+    </row>
+    <row r="6" ht="21" customHeight="1">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B6" s="49" t="n">
+      <c r="B6" s="25" t="n">
         <v>46305</v>
       </c>
-      <c r="C6" s="51" t="n"/>
-      <c r="D6" s="51" t="n"/>
-      <c r="E6" s="51" t="n"/>
-      <c r="F6" s="51" t="n"/>
-      <c r="G6" s="50" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="44" t="inlineStr">
+      <c r="C6" s="21" t="n"/>
+      <c r="D6" s="21" t="n"/>
+      <c r="E6" s="21" t="n"/>
+      <c r="F6" s="21" t="n"/>
+      <c r="G6" s="17" t="n"/>
+    </row>
+    <row r="7" ht="21" customHeight="1">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>Requirement</t>
         </is>
       </c>
-      <c r="B7" s="41" t="inlineStr">
+      <c r="B7" s="24" t="inlineStr">
         <is>
           <t>None (no dependencies)</t>
         </is>
       </c>
-      <c r="C7" s="51" t="n"/>
-      <c r="D7" s="51" t="n"/>
-      <c r="E7" s="51" t="n"/>
-      <c r="F7" s="51" t="n"/>
-      <c r="G7" s="50" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="43" t="inlineStr">
+      <c r="C7" s="21" t="n"/>
+      <c r="D7" s="21" t="n"/>
+      <c r="E7" s="21" t="n"/>
+      <c r="F7" s="21" t="n"/>
+      <c r="G7" s="17" t="n"/>
+    </row>
+    <row r="11" ht="21" customHeight="1">
+      <c r="A11" s="20" t="inlineStr">
         <is>
           <t>TestCaseID</t>
         </is>
       </c>
-      <c r="B11" s="43" t="inlineStr">
+      <c r="B11" s="20" t="inlineStr">
         <is>
           <t>Function Under Test</t>
         </is>
       </c>
-      <c r="C11" s="43" t="inlineStr">
+      <c r="C11" s="20" t="inlineStr">
         <is>
           <t>TestData</t>
         </is>
       </c>
-      <c r="D11" s="43" t="inlineStr">
+      <c r="D11" s="20" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="E11" s="43" t="inlineStr">
+      <c r="E11" s="20" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="F11" s="43" t="inlineStr">
+      <c r="F11" s="20" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="G11" s="43" t="inlineStr">
+      <c r="G11" s="20" t="inlineStr">
         <is>
           <t>DefectID</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="43" t="inlineStr">
+    <row r="12" ht="36" customHeight="1">
+      <c r="A12" s="20" t="inlineStr">
         <is>
           <t>TC01</t>
         </is>
       </c>
-      <c r="B12" s="43" t="inlineStr">
+      <c r="B12" s="20" t="inlineStr">
         <is>
           <t>execute</t>
         </is>
       </c>
-      <c r="C12" s="46" t="inlineStr">
+      <c r="C12" s="22" t="inlineStr">
         <is>
           <t>NoneCommand().execute()</t>
         </is>
       </c>
-      <c r="D12" s="46" t="inlineStr">
+      <c r="D12" s="22" t="inlineStr">
         <is>
           <t>no exception, no interaction</t>
         </is>
       </c>
-      <c r="E12" s="43" t="n"/>
-      <c r="F12" s="43" t="n"/>
-      <c r="G12" s="43" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="43" t="inlineStr">
+      <c r="E12" s="15" t="inlineStr">
+        <is>
+          <t>execute() throws nothing and touches no collaborator</t>
+        </is>
+      </c>
+      <c r="F12" s="20" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G12" s="20" t="n"/>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="20" t="inlineStr">
         <is>
           <t>TC02</t>
         </is>
       </c>
-      <c r="B13" s="43" t="inlineStr">
+      <c r="B13" s="20" t="inlineStr">
         <is>
           <t>getRecordedAction</t>
         </is>
       </c>
-      <c r="C13" s="46" t="inlineStr">
+      <c r="C13" s="22" t="inlineStr">
         <is>
           <t>any instance</t>
         </is>
       </c>
-      <c r="D13" s="46" t="inlineStr">
+      <c r="D13" s="22" t="inlineStr">
         <is>
           <t>ActionType.NONE</t>
         </is>
       </c>
-      <c r="E13" s="43" t="n"/>
-      <c r="F13" s="43" t="n"/>
-      <c r="G13" s="43" t="n"/>
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>ActionType.NONE</t>
+        </is>
+      </c>
+      <c r="F13" s="20" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G13" s="20" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -2122,261 +2109,300 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A3:G16"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.4"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="46" customWidth="1" min="3" max="3"/>
-    <col width="46" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="46" customWidth="1" min="3" max="4"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="3">
-      <c r="A3" s="44" t="inlineStr">
+    <row r="3" ht="21" customHeight="1">
+      <c r="A3" s="9" t="inlineStr">
         <is>
           <t>Project Name</t>
         </is>
       </c>
-      <c r="B3" s="41" t="inlineStr">
+      <c r="B3" s="24" t="inlineStr">
         <is>
           <t>Eternal Crash2</t>
         </is>
       </c>
-      <c r="C3" s="51" t="n"/>
-      <c r="D3" s="51" t="n"/>
-      <c r="E3" s="51" t="n"/>
-      <c r="F3" s="51" t="n"/>
-      <c r="G3" s="50" t="n"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="44" t="inlineStr">
+      <c r="C3" s="21" t="n"/>
+      <c r="D3" s="21" t="n"/>
+      <c r="E3" s="21" t="n"/>
+      <c r="F3" s="21" t="n"/>
+      <c r="G3" s="17" t="n"/>
+    </row>
+    <row r="4" ht="21" customHeight="1">
+      <c r="A4" s="9" t="inlineStr">
         <is>
           <t>SystemUnderTest/Class under Test</t>
         </is>
       </c>
-      <c r="B4" s="41" t="inlineStr">
+      <c r="B4" s="24" t="inlineStr">
         <is>
           <t>CommandFactory</t>
         </is>
       </c>
-      <c r="C4" s="51" t="n"/>
-      <c r="D4" s="51" t="n"/>
-      <c r="E4" s="51" t="n"/>
-      <c r="F4" s="51" t="n"/>
-      <c r="G4" s="50" t="n"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="44" t="inlineStr">
+      <c r="C4" s="21" t="n"/>
+      <c r="D4" s="21" t="n"/>
+      <c r="E4" s="21" t="n"/>
+      <c r="F4" s="21" t="n"/>
+      <c r="G4" s="17" t="n"/>
+    </row>
+    <row r="5" ht="21" customHeight="1">
+      <c r="A5" s="9" t="inlineStr">
         <is>
           <t>Environment</t>
         </is>
       </c>
-      <c r="B5" s="41" t="inlineStr">
-        <is>
-          <t>Window 11, java version "1.8.0_503" , Junit 5</t>
-        </is>
-      </c>
-      <c r="C5" s="51" t="n"/>
-      <c r="D5" s="51" t="n"/>
-      <c r="E5" s="51" t="n"/>
-      <c r="F5" s="51" t="n"/>
-      <c r="G5" s="50" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="44" t="inlineStr">
+      <c r="B5" s="24" t="inlineStr">
+        <is>
+          <t>Window 11, java version "17.0.12" , Junit 5</t>
+        </is>
+      </c>
+      <c r="C5" s="21" t="n"/>
+      <c r="D5" s="21" t="n"/>
+      <c r="E5" s="21" t="n"/>
+      <c r="F5" s="21" t="n"/>
+      <c r="G5" s="17" t="n"/>
+    </row>
+    <row r="6" ht="21" customHeight="1">
+      <c r="A6" s="9" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B6" s="49" t="n">
+      <c r="B6" s="25" t="n">
         <v>46305</v>
       </c>
-      <c r="C6" s="51" t="n"/>
-      <c r="D6" s="51" t="n"/>
-      <c r="E6" s="51" t="n"/>
-      <c r="F6" s="51" t="n"/>
-      <c r="G6" s="50" t="n"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="44" t="inlineStr">
+      <c r="C6" s="21" t="n"/>
+      <c r="D6" s="21" t="n"/>
+      <c r="E6" s="21" t="n"/>
+      <c r="F6" s="21" t="n"/>
+      <c r="G6" s="17" t="n"/>
+    </row>
+    <row r="7" ht="21" customHeight="1">
+      <c r="A7" s="9" t="inlineStr">
         <is>
           <t>Requirement</t>
         </is>
       </c>
-      <c r="B7" s="41" t="inlineStr">
+      <c r="B7" s="24" t="inlineStr">
         <is>
           <t>Mock CityService, ArmyService, GameEventRepository; real City/Game</t>
         </is>
       </c>
-      <c r="C7" s="51" t="n"/>
-      <c r="D7" s="51" t="n"/>
-      <c r="E7" s="51" t="n"/>
-      <c r="F7" s="51" t="n"/>
-      <c r="G7" s="50" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="43" t="inlineStr">
+      <c r="C7" s="21" t="n"/>
+      <c r="D7" s="21" t="n"/>
+      <c r="E7" s="21" t="n"/>
+      <c r="F7" s="21" t="n"/>
+      <c r="G7" s="17" t="n"/>
+    </row>
+    <row r="11" ht="21" customHeight="1">
+      <c r="A11" s="20" t="inlineStr">
         <is>
           <t>TestCaseID</t>
         </is>
       </c>
-      <c r="B11" s="43" t="inlineStr">
+      <c r="B11" s="20" t="inlineStr">
         <is>
           <t>Function Under Test</t>
         </is>
       </c>
-      <c r="C11" s="43" t="inlineStr">
+      <c r="C11" s="20" t="inlineStr">
         <is>
           <t>TestData</t>
         </is>
       </c>
-      <c r="D11" s="43" t="inlineStr">
+      <c r="D11" s="20" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="E11" s="43" t="inlineStr">
+      <c r="E11" s="20" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="F11" s="43" t="inlineStr">
+      <c r="F11" s="20" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="G11" s="43" t="inlineStr">
+      <c r="G11" s="20" t="inlineStr">
         <is>
           <t>DefectID</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="43" t="inlineStr">
+    <row r="12" ht="18" customHeight="1">
+      <c r="A12" s="20" t="inlineStr">
         <is>
           <t>TC01</t>
         </is>
       </c>
-      <c r="B12" s="43" t="inlineStr">
+      <c r="B12" s="20" t="inlineStr">
         <is>
           <t>createCommand</t>
         </is>
       </c>
-      <c r="C12" s="46" t="inlineStr">
+      <c r="C12" s="22" t="inlineStr">
         <is>
           <t>requestedAction = PRODUCE_FOOD</t>
         </is>
       </c>
-      <c r="D12" s="46" t="inlineStr">
+      <c r="D12" s="22" t="inlineStr">
         <is>
           <t>returns ProduceFoodCommand</t>
         </is>
       </c>
-      <c r="E12" s="43" t="n"/>
-      <c r="F12" s="43" t="n"/>
-      <c r="G12" s="43" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="43" t="inlineStr">
+      <c r="E12" s="15" t="inlineStr">
+        <is>
+          <t>ProduceFoodCommand instance</t>
+        </is>
+      </c>
+      <c r="F12" s="20" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G12" s="20" t="n"/>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="A13" s="20" t="inlineStr">
         <is>
           <t>TC02</t>
         </is>
       </c>
-      <c r="B13" s="43" t="inlineStr">
+      <c r="B13" s="20" t="inlineStr">
         <is>
           <t>createCommand</t>
         </is>
       </c>
-      <c r="C13" s="46" t="inlineStr">
+      <c r="C13" s="22" t="inlineStr">
         <is>
           <t>requestedAction = RECRUIT_SOLDIERS</t>
         </is>
       </c>
-      <c r="D13" s="46" t="inlineStr">
+      <c r="D13" s="22" t="inlineStr">
         <is>
           <t>returns RecruitSoldiersCommand</t>
         </is>
       </c>
-      <c r="E13" s="43" t="n"/>
-      <c r="F13" s="43" t="n"/>
-      <c r="G13" s="43" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="43" t="inlineStr">
+      <c r="E13" s="15" t="inlineStr">
+        <is>
+          <t>RecruitSoldiersCommand instance</t>
+        </is>
+      </c>
+      <c r="F13" s="20" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G13" s="20" t="n"/>
+    </row>
+    <row r="14" ht="36" customHeight="1">
+      <c r="A14" s="20" t="inlineStr">
         <is>
           <t>TC03</t>
         </is>
       </c>
-      <c r="B14" s="43" t="inlineStr">
+      <c r="B14" s="20" t="inlineStr">
         <is>
           <t>createCommand</t>
         </is>
       </c>
-      <c r="C14" s="46" t="inlineStr">
+      <c r="C14" s="22" t="inlineStr">
         <is>
           <t>requestedAction = SEND_ARMY, targetCityId 20, soldierCount 20</t>
         </is>
       </c>
-      <c r="D14" s="46" t="inlineStr">
+      <c r="D14" s="22" t="inlineStr">
         <is>
           <t>returns SendArmyCommand</t>
         </is>
       </c>
-      <c r="E14" s="43" t="n"/>
-      <c r="F14" s="43" t="n"/>
-      <c r="G14" s="43" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="43" t="inlineStr">
+      <c r="E14" s="15" t="inlineStr">
+        <is>
+          <t>SendArmyCommand instance</t>
+        </is>
+      </c>
+      <c r="F14" s="20" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G14" s="20" t="n"/>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="A15" s="20" t="inlineStr">
         <is>
           <t>TC04</t>
         </is>
       </c>
-      <c r="B15" s="43" t="inlineStr">
+      <c r="B15" s="20" t="inlineStr">
         <is>
           <t>createCommand</t>
         </is>
       </c>
-      <c r="C15" s="46" t="inlineStr">
+      <c r="C15" s="22" t="inlineStr">
         <is>
           <t>requestedAction = NONE</t>
         </is>
       </c>
-      <c r="D15" s="46" t="inlineStr">
+      <c r="D15" s="22" t="inlineStr">
         <is>
           <t>returns NoneCommand</t>
         </is>
       </c>
-      <c r="E15" s="43" t="n"/>
-      <c r="F15" s="43" t="n"/>
-      <c r="G15" s="43" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="43" t="inlineStr">
+      <c r="E15" s="15" t="inlineStr">
+        <is>
+          <t>NoneCommand instance</t>
+        </is>
+      </c>
+      <c r="F15" s="20" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G15" s="20" t="n"/>
+    </row>
+    <row r="16" ht="36" customHeight="1">
+      <c r="A16" s="20" t="inlineStr">
         <is>
           <t>TC05</t>
         </is>
       </c>
-      <c r="B16" s="43" t="inlineStr">
+      <c r="B16" s="20" t="inlineStr">
         <is>
           <t>createCommand</t>
         </is>
       </c>
-      <c r="C16" s="46" t="inlineStr">
+      <c r="C16" s="22" t="inlineStr">
         <is>
           <t>requestedAction = null</t>
         </is>
       </c>
-      <c r="D16" s="46" t="inlineStr">
+      <c r="D16" s="22" t="inlineStr">
         <is>
           <t>returns NoneCommand</t>
         </is>
       </c>
-      <c r="E16" s="43" t="n"/>
-      <c r="F16" s="43" t="n"/>
-      <c r="G16" s="43" t="n"/>
+      <c r="E16" s="15" t="inlineStr">
+        <is>
+          <t>NoneCommand instance for a null requestedAction</t>
+        </is>
+      </c>
+      <c r="F16" s="20" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+      <c r="G16" s="20" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="5">

</xml_diff>